<commit_message>
Publish course viewer from mmejza/MKT495_repo@758aae48567c63e68a991350871adec6f89dc943
</commit_message>
<xml_diff>
--- a/breakouts/files/class-03-report-out.xlsx
+++ b/breakouts/files/class-03-report-out.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rb8836b1c6b8b4f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Process" sheetId="2" r:id="Rce27f1893fc8410a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Focus Group Design" sheetId="3" r:id="R46a6896811b54a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positioning Plans" sheetId="4" r:id="R7fcafc6ffeaa4143"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R6c2a63221d8b41fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Process" sheetId="2" r:id="Redb1961aa45946cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Focus Group Design" sheetId="3" r:id="R42da290a20824281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positioning Plans" sheetId="4" r:id="R3b19d9a0862141a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -54,8 +54,31 @@
       <x:color rgb="FF6F0000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF8B0000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +108,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC00000"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4E4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF262626"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -127,7 +175,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -181,6 +229,52 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -514,7 +608,7 @@
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" s="23" t="str">
-        <x:v>3. Develop complete Family Connection and Clever Cooking positioning plans.</x:v>
+        <x:v>3. Develop complete Family Connection and Clever Cooking positioning plans without AI assistance.</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
         <x:v>3. Develop complete Family Connection and Clever Cooking positioning plans.</x:v>
@@ -606,7 +700,7 @@
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>Recommended focus-group design principle</x:v>
+        <x:v>Logic behind the four focus groups</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>Recommended focus-group design principle</x:v>
@@ -618,7 +712,7 @@
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Preferred positioning concept and why</x:v>
+        <x:v>Chosen positioning concept</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>Preferred positioning concept and why</x:v>
@@ -627,6 +721,30 @@
       <x:c r="D19" s="19"/>
       <x:c r="E19" s="19"/>
       <x:c r="F19" s="19"/>
+    </x:row>
+    <x:row r="20" ht="58" customHeight="1">
+      <x:c r="A20" s="34" t="str">
+        <x:v>Strongest case evidence supporting the choice</x:v>
+      </x:c>
+      <x:c r="B20" s="34" t="str">
+        <x:v>Preferred positioning concept and why</x:v>
+      </x:c>
+      <x:c r="C20" s="39"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="39"/>
+      <x:c r="F20" s="39"/>
+    </x:row>
+    <x:row r="21" ht="58" customHeight="1">
+      <x:c r="A21" s="34" t="str">
+        <x:v>AI judgment: suggestion → concern → change → why</x:v>
+      </x:c>
+      <x:c r="B21" s="34" t="str">
+        <x:v>Preferred positioning concept and why</x:v>
+      </x:c>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="39"/>
+      <x:c r="F21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -646,6 +764,10 @@
     <x:mergeCell ref="C18:F18"/>
     <x:mergeCell ref="A19:B19"/>
     <x:mergeCell ref="C19:F19"/>
+    <x:mergeCell ref="A20:B20"/>
+    <x:mergeCell ref="C20:F20"/>
+    <x:mergeCell ref="A21:B21"/>
+    <x:mergeCell ref="C21:F21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -659,6 +781,7 @@
     <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -674,10 +797,11 @@
       <x:c r="D1" s="3" t="str">
         <x:v>Four-Step Research Process</x:v>
       </x:c>
+      <x:c r="E1" s="42"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="29" t="str">
-        <x:v>For each step, distinguish the activity, information objective, and resulting insight.</x:v>
+        <x:v>For each stage, identify what occurred, why it was done, what was learned, and the decision or next step it enabled. AI may assist, but identify where it may confuse an activity, finding, insight, or recommendation.</x:v>
       </x:c>
       <x:c r="B2" s="29" t="str">
         <x:v>For each step, distinguish the activity, information objective, and resulting insight.</x:v>
@@ -688,6 +812,7 @@
       <x:c r="D2" s="29" t="str">
         <x:v>For each step, distinguish the activity, information objective, and resulting insight.</x:v>
       </x:c>
+      <x:c r="E2" s="46"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="9" t="str">
@@ -702,6 +827,9 @@
       <x:c r="D4" s="9" t="str">
         <x:v>Key Findings / Outcomes</x:v>
       </x:c>
+      <x:c r="E4" s="51" t="str">
+        <x:v>Decision / Next Step Enabled</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="72" customHeight="1">
       <x:c r="A5" s="14" t="str">
@@ -712,6 +840,7 @@
       </x:c>
       <x:c r="C5" s="19"/>
       <x:c r="D5" s="19"/>
+      <x:c r="E5" s="39"/>
     </x:row>
     <x:row r="6" ht="72" customHeight="1">
       <x:c r="A6" s="14" t="str">
@@ -720,6 +849,7 @@
       <x:c r="B6" s="19"/>
       <x:c r="C6" s="19"/>
       <x:c r="D6" s="19"/>
+      <x:c r="E6" s="39"/>
     </x:row>
     <x:row r="7" ht="72" customHeight="1">
       <x:c r="A7" s="14" t="str">
@@ -728,6 +858,7 @@
       <x:c r="B7" s="19"/>
       <x:c r="C7" s="19"/>
       <x:c r="D7" s="19"/>
+      <x:c r="E7" s="39"/>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
       <x:c r="A8" s="14" t="str">
@@ -736,6 +867,7 @@
       <x:c r="B8" s="19"/>
       <x:c r="C8" s="19"/>
       <x:c r="D8" s="19"/>
+      <x:c r="E8" s="39"/>
     </x:row>
     <x:row r="9" ht="72" customHeight="1">
       <x:c r="A9" s="14" t="str">
@@ -744,6 +876,7 @@
       <x:c r="B9" s="19"/>
       <x:c r="C9" s="19"/>
       <x:c r="D9" s="19"/>
+      <x:c r="E9" s="39"/>
     </x:row>
     <x:row r="10" ht="72" customHeight="1">
       <x:c r="A10" s="14" t="str">
@@ -752,11 +885,23 @@
       <x:c r="B10" s="19"/>
       <x:c r="C10" s="19"/>
       <x:c r="D10" s="19"/>
+      <x:c r="E10" s="39"/>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="34" t="str">
+        <x:v>AI check: Where might AI confuse an activity, finding, insight, or recommendation?</x:v>
+      </x:c>
+      <x:c r="B11" s="34"/>
+      <x:c r="C11" s="39"/>
+      <x:c r="D11" s="39"/>
+      <x:c r="E11" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:D1"/>
-    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A11:B11"/>
+    <x:mergeCell ref="C11:E11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -771,6 +916,7 @@
     <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="31" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -789,10 +935,11 @@
       <x:c r="E1" s="3" t="str">
         <x:v>Four Focus Groups</x:v>
       </x:c>
+      <x:c r="F1" s="42"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="29" t="str">
-        <x:v>Use Exhibit 3 variables to create complementary groups and explain the information value of each.</x:v>
+        <x:v>Use Exhibit 3 variables to create complementary groups. AI may propose a design; identify its weakest element, revise it, ask AI to critique the revision, and decide which criticisms to accept or reject.</x:v>
       </x:c>
       <x:c r="B2" s="29" t="str">
         <x:v>Use Exhibit 3 variables to create complementary groups and explain the information value of each.</x:v>
@@ -806,6 +953,7 @@
       <x:c r="E2" s="29" t="str">
         <x:v>Use Exhibit 3 variables to create complementary groups and explain the information value of each.</x:v>
       </x:c>
+      <x:c r="F2" s="46"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="9" t="str">
@@ -822,6 +970,9 @@
       </x:c>
       <x:c r="E4" s="9" t="str">
         <x:v>Why Interview This Group?</x:v>
+      </x:c>
+      <x:c r="F4" s="51" t="str">
+        <x:v>What This Group Adds</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="78" customHeight="1">
@@ -832,6 +983,7 @@
       <x:c r="C5" s="19"/>
       <x:c r="D5" s="19"/>
       <x:c r="E5" s="19"/>
+      <x:c r="F5" s="39"/>
     </x:row>
     <x:row r="6" ht="78" customHeight="1">
       <x:c r="A6" s="14" t="str">
@@ -841,6 +993,7 @@
       <x:c r="C6" s="19"/>
       <x:c r="D6" s="19"/>
       <x:c r="E6" s="19"/>
+      <x:c r="F6" s="39"/>
     </x:row>
     <x:row r="7" ht="78" customHeight="1">
       <x:c r="A7" s="14" t="str">
@@ -850,6 +1003,7 @@
       <x:c r="C7" s="19"/>
       <x:c r="D7" s="19"/>
       <x:c r="E7" s="19"/>
+      <x:c r="F7" s="39"/>
     </x:row>
     <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="14" t="str">
@@ -859,24 +1013,40 @@
       <x:c r="C8" s="19"/>
       <x:c r="D8" s="19"/>
       <x:c r="E8" s="19"/>
-    </x:row>
-    <x:row r="10" ht="84" customHeight="1">
-      <x:c r="A10" s="14" t="str">
+      <x:c r="F8" s="39"/>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="34" t="str">
+        <x:v>What important customer variation does your design capture?</x:v>
+      </x:c>
+      <x:c r="B10" s="34" t="str">
         <x:v>How do the four groups work together to reveal behaviors, purchase triggers, unmet needs, benefits, and values?</x:v>
       </x:c>
-      <x:c r="B10" s="14" t="str">
+      <x:c r="C10" s="39"/>
+      <x:c r="D10" s="39"/>
+      <x:c r="E10" s="39"/>
+      <x:c r="F10" s="39"/>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="34" t="str">
+        <x:v>What important blind spot might remain?</x:v>
+      </x:c>
+      <x:c r="B11" s="34" t="str">
         <x:v>How do the four groups work together to reveal behaviors, purchase triggers, unmet needs, benefits, and values?</x:v>
       </x:c>
-      <x:c r="C10" s="19"/>
-      <x:c r="D10" s="19"/>
-      <x:c r="E10" s="19"/>
+      <x:c r="C11" s="39"/>
+      <x:c r="D11" s="39"/>
+      <x:c r="E11" s="39"/>
+      <x:c r="F11" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:E1"/>
-    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
     <x:mergeCell ref="A10:B10"/>
-    <x:mergeCell ref="C10:E10"/>
+    <x:mergeCell ref="C10:F10"/>
+    <x:mergeCell ref="A11:B11"/>
+    <x:mergeCell ref="C11:F11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -904,7 +1074,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="29" t="str">
-        <x:v>Build each concept from attributes through functional and emotional benefits to a core value.</x:v>
+        <x:v>Complete Activity 3 without AI. Build each concept from attributes through functional and emotional benefits to a core value, then develop the positioning and execution.</x:v>
       </x:c>
       <x:c r="B2" s="29" t="str">
         <x:v>Build each concept from attributes through functional and emotional benefits to a core value.</x:v>
@@ -926,102 +1096,132 @@
     </x:row>
     <x:row r="5" ht="52" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Brand name</x:v>
+        <x:v>Product attributes</x:v>
       </x:c>
       <x:c r="B5" s="19"/>
       <x:c r="C5" s="19"/>
     </x:row>
     <x:row r="6" ht="52" customHeight="1">
       <x:c r="A6" s="14" t="str">
-        <x:v>Positioning statement</x:v>
+        <x:v>Functional benefit</x:v>
       </x:c>
       <x:c r="B6" s="19"/>
       <x:c r="C6" s="19"/>
     </x:row>
     <x:row r="7" ht="52" customHeight="1">
       <x:c r="A7" s="14" t="str">
-        <x:v>Core belief / value</x:v>
+        <x:v>Personal or emotional benefit</x:v>
       </x:c>
       <x:c r="B7" s="19"/>
       <x:c r="C7" s="19"/>
     </x:row>
     <x:row r="8" ht="52" customHeight="1">
       <x:c r="A8" s="14" t="str">
-        <x:v>Personal or emotional benefit</x:v>
+        <x:v>Core belief / value</x:v>
       </x:c>
       <x:c r="B8" s="19"/>
       <x:c r="C8" s="19"/>
     </x:row>
     <x:row r="9" ht="52" customHeight="1">
       <x:c r="A9" s="14" t="str">
-        <x:v>Functional benefit</x:v>
+        <x:v>Positioning statement</x:v>
       </x:c>
       <x:c r="B9" s="19"/>
       <x:c r="C9" s="19"/>
     </x:row>
     <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>Product attributes</x:v>
+        <x:v>Form(s)</x:v>
       </x:c>
       <x:c r="B10" s="19"/>
       <x:c r="C10" s="19"/>
     </x:row>
     <x:row r="11" ht="52" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>Form(s)</x:v>
+        <x:v>Flavor(s) / flavoring</x:v>
       </x:c>
       <x:c r="B11" s="19"/>
       <x:c r="C11" s="19"/>
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>Flavor(s) / flavoring</x:v>
+        <x:v>Packaging</x:v>
       </x:c>
       <x:c r="B12" s="19"/>
       <x:c r="C12" s="19"/>
     </x:row>
     <x:row r="13" ht="52" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>Other variation(s)</x:v>
+        <x:v>In-store merchandising</x:v>
       </x:c>
       <x:c r="B13" s="19"/>
       <x:c r="C13" s="19"/>
     </x:row>
     <x:row r="14" ht="52" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>Packaging</x:v>
+        <x:v>Advertising tagline</x:v>
       </x:c>
       <x:c r="B14" s="19"/>
       <x:c r="C14" s="19"/>
     </x:row>
     <x:row r="15" ht="52" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>In-store merchandising</x:v>
+        <x:v>Strategic logic</x:v>
       </x:c>
       <x:c r="B15" s="19"/>
       <x:c r="C15" s="19"/>
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>Advertising tagline</x:v>
+        <x:v>Strongest supporting case evidence</x:v>
       </x:c>
       <x:c r="B16" s="19"/>
       <x:c r="C16" s="19"/>
     </x:row>
-    <x:row r="18" ht="72" customHeight="1">
-      <x:c r="A18" s="14" t="str">
+    <x:row r="18" ht="58" customHeight="1">
+      <x:c r="A18" s="34" t="str">
+        <x:v>Evaluation criteria for comparing the alternatives</x:v>
+      </x:c>
+      <x:c r="B18" s="34" t="str">
         <x:v>Which concept should Saxonville pursue, and what evidence supports that choice?</x:v>
       </x:c>
-      <x:c r="B18" s="14" t="str">
+      <x:c r="C18" s="39"/>
+    </x:row>
+    <x:row r="19" ht="58" customHeight="1">
+      <x:c r="A19" s="34" t="str">
+        <x:v>Which concept should Saxonville pursue, and why?</x:v>
+      </x:c>
+      <x:c r="B19" s="34" t="str">
         <x:v>Which concept should Saxonville pursue, and what evidence supports that choice?</x:v>
       </x:c>
-      <x:c r="C18" s="19"/>
+      <x:c r="C19" s="39"/>
+    </x:row>
+    <x:row r="20" ht="58" customHeight="1">
+      <x:c r="A20" s="34" t="str">
+        <x:v>Strongest argument for the position you rejected</x:v>
+      </x:c>
+      <x:c r="B20" s="34" t="str">
+        <x:v>Which concept should Saxonville pursue, and what evidence supports that choice?</x:v>
+      </x:c>
+      <x:c r="C20" s="39"/>
+    </x:row>
+    <x:row r="21" ht="58" customHeight="1">
+      <x:c r="A21" s="34" t="str">
+        <x:v>What additional evidence could reverse your decision?</x:v>
+      </x:c>
+      <x:c r="B21" s="34" t="str">
+        <x:v>Which concept should Saxonville pursue, and what evidence supports that choice?</x:v>
+      </x:c>
+      <x:c r="C21" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:C1"/>
     <x:mergeCell ref="A2:C2"/>
     <x:mergeCell ref="A18:B18"/>
+    <x:mergeCell ref="A19:B19"/>
+    <x:mergeCell ref="A20:B20"/>
+    <x:mergeCell ref="A21:B21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>